<commit_message>
docs: update supplier template with multi-category support (pipe-separated)
</commit_message>
<xml_diff>
--- a/public/templates/TEMPLATE_Supplier.xlsx
+++ b/public/templates/TEMPLATE_Supplier.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Supplier" sheetId="1" r:id="rId1"/>
+    <sheet name="Suppliers" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,24 +397,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:H22"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="22.83203125" customWidth="1"/>
-    <col min="7" max="7" width="22.83203125" customWidth="1"/>
-    <col min="8" max="8" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="25.83203125" customWidth="1"/>
+    <col min="2" max="2" width="18.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="45.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>ชื่อ Supplier/บริษัท*</v>
+        <v>ชื่อผู้จำหน่าย</v>
       </c>
       <c r="B1" t="str">
-        <v>ชื่อผู้ติดต่อ</v>
+        <v>ผู้ติดต่อ</v>
       </c>
       <c r="C1" t="str">
         <v>เบอร์โทร</v>
@@ -423,13 +423,13 @@
         <v>อีเมล</v>
       </c>
       <c r="E1" t="str">
-        <v>หมวดสินค้า</v>
+        <v>ที่อยู่</v>
       </c>
       <c r="F1" t="str">
+        <v>ประเภทสินค้า (แยก | ถ้าหลายอย่าง)</v>
+      </c>
+      <c r="G1" t="str">
         <v>เงื่อนไขการชำระ</v>
-      </c>
-      <c r="G1" t="str">
-        <v>ที่อยู่</v>
       </c>
       <c r="H1" t="str">
         <v>หมายเหตุ</v>
@@ -437,51 +437,51 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>ชื่อบริษัทหรือร้านค้า</v>
+        <v>บริษัท กระจกไทย จำกัด</v>
       </c>
       <c r="B2" t="str">
-        <v>ชื่อ-นามสกุล</v>
+        <v>สมชัย ทดสอบ</v>
       </c>
       <c r="C2" t="str">
-        <v>เบอร์โทร</v>
+        <v>089-1234567</v>
       </c>
       <c r="D2" t="str">
-        <v>อีเมลติดต่อ</v>
+        <v>contact@glass.co.th</v>
       </c>
       <c r="E2" t="str">
-        <v>เช่น กระจก / อลูมิเนียม / อุปกรณ์</v>
+        <v>123 ซอย 5 บางนา</v>
       </c>
       <c r="F2" t="str">
-        <v>เช่น 30 วัน / เงินสด</v>
+        <v>กระจก|ซิลิโคน/ยาง</v>
       </c>
       <c r="G2" t="str">
-        <v>ที่อยู่</v>
+        <v>30 วัน</v>
       </c>
       <c r="H2" t="str">
-        <v/>
+        <v>บริษัทชั้นหนึ่ง</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>บริษัท กระจกไทย จำกัด</v>
+        <v/>
       </c>
       <c r="B3" t="str">
-        <v>คุณประสิทธิ์ แก้วใส</v>
+        <v/>
       </c>
       <c r="C3" t="str">
-        <v>02-456-7890</v>
+        <v/>
       </c>
       <c r="D3" t="str">
-        <v>sales@thaiglass.com</v>
+        <v/>
       </c>
       <c r="E3" t="str">
-        <v>กระจก</v>
+        <v/>
       </c>
       <c r="F3" t="str">
-        <v>30 วัน</v>
+        <v/>
       </c>
       <c r="G3" t="str">
-        <v>ลาดพร้าว กรุงเทพฯ</v>
+        <v/>
       </c>
       <c r="H3" t="str">
         <v/>
@@ -489,33 +489,501 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ห้างอลูมิเนียมสยาม</v>
+        <v/>
       </c>
       <c r="B4" t="str">
-        <v>คุณมานะ แข็งแกร่ง</v>
+        <v/>
       </c>
       <c r="C4" t="str">
-        <v>081-987-6543</v>
+        <v/>
       </c>
       <c r="D4" t="str">
         <v/>
       </c>
       <c r="E4" t="str">
-        <v>อลูมิเนียม/เหล็ก</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>เงินสด</v>
+        <v/>
       </c>
       <c r="G4" t="str">
-        <v>สมุทรปราการ</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>ราคาดี</v>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v/>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+      <c r="H5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v/>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+      <c r="H6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v/>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v/>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v/>
+      </c>
+      <c r="B9" t="str">
+        <v/>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v/>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v/>
+      </c>
+      <c r="B10" t="str">
+        <v/>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v/>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+      <c r="F10" t="str">
+        <v/>
+      </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v/>
+      </c>
+      <c r="B11" t="str">
+        <v/>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v/>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+      <c r="F11" t="str">
+        <v/>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v/>
+      </c>
+      <c r="B12" t="str">
+        <v/>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+      <c r="F12" t="str">
+        <v/>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v/>
+      </c>
+      <c r="B13" t="str">
+        <v/>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v/>
+      </c>
+      <c r="B14" t="str">
+        <v/>
+      </c>
+      <c r="C14" t="str">
+        <v/>
+      </c>
+      <c r="D14" t="str">
+        <v/>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+      <c r="F14" t="str">
+        <v/>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v/>
+      </c>
+      <c r="B15" t="str">
+        <v/>
+      </c>
+      <c r="C15" t="str">
+        <v/>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+      <c r="F15" t="str">
+        <v/>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v/>
+      </c>
+      <c r="B16" t="str">
+        <v/>
+      </c>
+      <c r="C16" t="str">
+        <v/>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v/>
+      </c>
+      <c r="F16" t="str">
+        <v/>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v/>
+      </c>
+      <c r="B17" t="str">
+        <v/>
+      </c>
+      <c r="C17" t="str">
+        <v/>
+      </c>
+      <c r="D17" t="str">
+        <v/>
+      </c>
+      <c r="E17" t="str">
+        <v/>
+      </c>
+      <c r="F17" t="str">
+        <v/>
+      </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+      <c r="B18" t="str">
+        <v/>
+      </c>
+      <c r="C18" t="str">
+        <v/>
+      </c>
+      <c r="D18" t="str">
+        <v/>
+      </c>
+      <c r="E18" t="str">
+        <v/>
+      </c>
+      <c r="F18" t="str">
+        <v/>
+      </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v/>
+      </c>
+      <c r="B19" t="str">
+        <v/>
+      </c>
+      <c r="C19" t="str">
+        <v/>
+      </c>
+      <c r="D19" t="str">
+        <v/>
+      </c>
+      <c r="E19" t="str">
+        <v/>
+      </c>
+      <c r="F19" t="str">
+        <v/>
+      </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v/>
+      </c>
+      <c r="B20" t="str">
+        <v/>
+      </c>
+      <c r="C20" t="str">
+        <v/>
+      </c>
+      <c r="D20" t="str">
+        <v/>
+      </c>
+      <c r="E20" t="str">
+        <v/>
+      </c>
+      <c r="F20" t="str">
+        <v/>
+      </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v/>
+      </c>
+      <c r="B21" t="str">
+        <v/>
+      </c>
+      <c r="C21" t="str">
+        <v/>
+      </c>
+      <c r="D21" t="str">
+        <v/>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+      <c r="F21" t="str">
+        <v/>
+      </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v/>
+      </c>
+      <c r="B22" t="str">
+        <v/>
+      </c>
+      <c r="C22" t="str">
+        <v/>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+      <c r="F22" t="str">
+        <v/>
+      </c>
+      <c r="G22" t="str">
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H22"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>